<commit_message>
Add NIST reference (800-53B baselines, 800-53A assessment), solution walkthroughs, signature metadata; keep build scripts local
</commit_message>
<xml_diff>
--- a/episode-01-csf/meridian-csf-profile-BLANK.xlsx
+++ b/episode-01-csf/meridian-csf-profile-BLANK.xlsx
@@ -1491,6 +1491,14 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LField Notes Lab  -  fictional, for teaching&amp;COmar Mahdy&amp;R&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1608,5 +1616,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LField Notes Lab  -  fictional, for teaching&amp;COmar Mahdy&amp;R&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>